<commit_message>
feat: support BOF spec-only charts (V10.10)
</commit_message>
<xml_diff>
--- a/app-assets/bof-boxplot/BOF箱线图分析案例数据.xlsx
+++ b/app-assets/bof-boxplot/BOF箱线图分析案例数据.xlsx
@@ -11,8 +11,7 @@
     <sheet name="使用说明" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Data" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Spec" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="BinPlot" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="HL SN" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="HL SN" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -24,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
   <si>
     <r>
       <rPr>
@@ -207,6 +206,53 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">HL SN</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Linux Libertine G"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">填写需要突出显示的 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Linux Libertine G"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，必须存在于 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Linux Libertine G"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">BinPlot</t>
   </si>
   <si>
@@ -216,78 +262,106 @@
         <rFont val="Linux Libertine G"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">定义每个 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">BinType </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">的连续区间、名称与颜色。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">HL SN</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">填写需要突出显示的 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">，必须存在于 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Data</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">注意</t>
-  </si>
-  <si>
-    <t xml:space="preserve">本案例仅用于功能演示，不代表正式产品规范。</t>
+      <t xml:space="preserve">可选；本案例不提供。缺少时按 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Spec </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Linux Libertine G"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">的 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">USL/LSL </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Linux Libertine G"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">画上下限，不绘制 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Bin </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Linux Libertine G"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">色带。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">本案例</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Linux Libertine G"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">不含 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BinPlot </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Linux Libertine G"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">工作表，图表仅显示 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Spec </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Linux Libertine G"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">上下限；案例数据不代表正式产品规范。</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">No</t>
@@ -527,30 +601,6 @@
   </si>
   <si>
     <t xml:space="preserve">平面度</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BInName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Color</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low</t>
-  </si>
-  <si>
-    <t xml:space="preserve">绿色</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">黄色</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High</t>
-  </si>
-  <si>
-    <t xml:space="preserve">橙色</t>
   </si>
 </sst>
 </file>
@@ -1425,151 +1475,6 @@
     <tabColor rgb="FF315F85"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="5.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="5.71"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="10" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="D2" s="10" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="10" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D3" s="10" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" s="10" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="10" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <tabColor rgb="FF315F85"/>
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>

</xml_diff>